<commit_message>
feat(compiler): settings sheet, build configuration, any locale, query levels
- Inputs, outputs and metadata come from a settings sheet of the workbook
  (key, value, description, meta_type); the executable lists them with --meta.
  --in/--out are removed.
- sheetc.toml (or --config) holds the build options; flags override the file.
- Locale: any BCP-47 tag, resolved from CLDR through ICU4X (separators, month
  and day names, date order) with a [locale] table to override; fixed at build
  time. --runtime-locale and the locale taint analysis are removed.
- --outputs declared|named|any decides what a caller may query at run time
  (--query RANGE, "$query" in the JSON); the program keeps progressively more.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011MRBtaN4HWRL7ovwpZgUes
</commit_message>
<xml_diff>
--- a/sheetrs-compiler/tests/assets/loan.xlsx
+++ b/sheetrs-compiler/tests/assets/loan.xlsx
@@ -9,6 +9,7 @@
   </bookViews>
   <sheets>
     <sheet name="Loan" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="settings" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
   <si>
     <t xml:space="preserve">Principal</t>
   </si>
@@ -59,6 +60,57 @@
   </si>
   <si>
     <t xml:space="preserve">Unused note</t>
+  </si>
+  <si>
+    <t xml:space="preserve">key</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">meta_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">output</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan!B8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Model version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">info</t>
   </si>
 </sst>
 </file>
@@ -6568,4 +6620,128 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="0" t="s">
+        <v>13</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="0" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" s="0" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="C2" s="0" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="0" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" s="0" t="s">
+        <v>1</v>
+      </c>
+      <c r="D3" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>2</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>6</v>
+      </c>
+      <c r="D5" s="0" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>3</v>
+      </c>
+      <c r="D6" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" s="0" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="0" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="0" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="0" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="0" t="s">
+        <v>28</v>
+      </c>
+      <c r="D9" s="0" t="s">
+        <v>29</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
refactor(compiler): aliases in the settings sheet, in-house collation, explicit locales
- Settings sheet: `key` is the JSON name, `value` the range (starting with the
  sheet, a sheet name or a defined name) or, for metadata, the literal.
- Collation: replace ICU4X with a table derived once from ICU (checked against
  it over 1.6 M random pairs for en/es, both strengths, plus a golden test).
  Comparison 138 -> 31 ns; runtime stub 3.97 -> 2.71 MB; sheetc 6.50 -> 4.04 MB.
- Locales: en and es built in; other regions and languages are stated in the
  [locale] table (fail-fast when something is missing) instead of derived.
- PROGRAM_VERSION back to 1: nothing was released with the earlier layout.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011MRBtaN4HWRL7ovwpZgUes
</commit_message>
<xml_diff>
--- a/sheetrs-compiler/tests/assets/loan.xlsx
+++ b/sheetrs-compiler/tests/assets/loan.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="39">
   <si>
     <t xml:space="preserve">Principal</t>
   </si>
@@ -74,19 +74,40 @@
     <t xml:space="preserve">meta_type</t>
   </si>
   <si>
+    <t xml:space="preserve">principal</t>
+  </si>
+  <si>
     <t xml:space="preserve">Loan!B1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Loan amount</t>
   </si>
   <si>
     <t xml:space="preserve">input</t>
   </si>
   <si>
+    <t xml:space="preserve">rate</t>
+  </si>
+  <si>
     <t xml:space="preserve">Loan!B2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">years</t>
   </si>
   <si>
     <t xml:space="preserve">Loan!B3</t>
   </si>
   <si>
+    <t xml:space="preserve">Term in years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">month</t>
+  </si>
+  <si>
     <t xml:space="preserve">Loan!B7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">payment</t>
   </si>
   <si>
     <t xml:space="preserve">Loan!B4</t>
@@ -95,7 +116,13 @@
     <t xml:space="preserve">output</t>
   </si>
   <si>
+    <t xml:space="preserve">interest</t>
+  </si>
+  <si>
     <t xml:space="preserve">Loan!B6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">balance</t>
   </si>
   <si>
     <t xml:space="preserve">Loan!B8</t>
@@ -6648,91 +6675,112 @@
       <c r="A2" s="0" t="s">
         <v>17</v>
       </c>
+      <c r="B2" s="0" t="s">
+        <v>18</v>
+      </c>
       <c r="C2" s="0" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D2" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="0" t="s">
-        <v>19</v>
+        <v>21</v>
+      </c>
+      <c r="B3" s="0" t="s">
+        <v>22</v>
       </c>
       <c r="C3" s="0" t="s">
         <v>1</v>
       </c>
       <c r="D3" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="0" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" s="0" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" s="0" t="s">
         <v>20</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>2</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="0" t="s">
-        <v>21</v>
+        <v>26</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>27</v>
       </c>
       <c r="C5" s="0" t="s">
         <v>6</v>
       </c>
       <c r="D5" s="0" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="0" t="s">
-        <v>22</v>
+        <v>28</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>29</v>
       </c>
       <c r="C6" s="0" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="0" t="s">
-        <v>24</v>
+        <v>31</v>
+      </c>
+      <c r="B7" s="0" t="s">
+        <v>32</v>
       </c>
       <c r="C7" s="0" t="s">
         <v>5</v>
       </c>
       <c r="D7" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="0" t="s">
-        <v>25</v>
+        <v>33</v>
+      </c>
+      <c r="B8" s="0" t="s">
+        <v>34</v>
       </c>
       <c r="C8" s="0" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="0" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="0" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B9" s="0" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="C9" s="0" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="D9" s="0" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>